<commit_message>
Fehler behoben in apply_clustering: Anstatt optimal_feature_set wurden alle Features für die Dendrogramme verwendet; Überarbeitung der Plots.
</commit_message>
<xml_diff>
--- a/data/naturverbundenheit_indices.xlsx
+++ b/data/naturverbundenheit_indices.xlsx
@@ -1,35 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Programmierung\Dierkes\evaluation_cluster_based\data\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C72095E9-8901-49B2-8E66-69FFE818867E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="4995" yWindow="6360" windowWidth="23580" windowHeight="12405" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet r:id="rId1" sheetId="1" name="Sheet1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
-    </ext>
-  </extLst>
+  <calcPr fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -108,13 +88,13 @@
     <t>Dominican Republic</t>
   </si>
   <si>
-    <t xml:space="preserve">Ecuador </t>
+    <t>Ecuador</t>
   </si>
   <si>
     <t>France</t>
   </si>
   <si>
-    <t xml:space="preserve">Germany </t>
+    <t>Germany</t>
   </si>
   <si>
     <t>India</t>
@@ -195,39 +175,22 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
+  <numFmts count="0"/>
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
-      <color rgb="FF000000"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="1"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Cambria"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
       <family val="2"/>
-      <charset val="1"/>
     </font>
     <font>
       <b/>
@@ -235,30 +198,20 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <charset val="1"/>
     </font>
     <font>
       <b/>
       <u/>
       <sz val="11"/>
-      <color rgb="FF0000FF"/>
+      <color rgb="FF0000ff"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="1"/>
     </font>
     <font>
       <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -269,7 +222,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -279,174 +232,129 @@
     </border>
     <border>
       <left style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </left>
       <right style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </right>
       <top style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFd9d9d9"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFd9d9d9"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFd9d9d9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFd9d9d9"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFD9D9D9"/>
+        <color rgb="FFd9d9d9"/>
       </left>
       <right style="thin">
-        <color rgb="FFD9D9D9"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFD9D9D9"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFD9D9D9"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFD9D9D9"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFD9D9D9"/>
+        <color rgb="FFd9d9d9"/>
       </right>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+  <cellXfs count="17">
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyProtection="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="4" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
-  <cellStyles count="3">
-    <cellStyle name="Link" xfId="1" builtinId="8"/>
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
-    <cellStyle name="Standard_Tabelle1" xfId="2" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
+  <cellStyles count="1">
+    <cellStyle xfId="0" builtinId="0" name="Normal"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="FF000000"/>
-      <rgbColor rgb="FFFFFFFF"/>
-      <rgbColor rgb="FFFF0000"/>
-      <rgbColor rgb="FF00FF00"/>
-      <rgbColor rgb="FF0000FF"/>
-      <rgbColor rgb="FFFFFF00"/>
-      <rgbColor rgb="FFFF00FF"/>
-      <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF008000"/>
-      <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FF808000"/>
-      <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FFC0C0C0"/>
-      <rgbColor rgb="FF808080"/>
-      <rgbColor rgb="FF9999FF"/>
-      <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFFFCC"/>
-      <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FF660066"/>
-      <rgbColor rgb="FFFF8080"/>
-      <rgbColor rgb="FF0066CC"/>
-      <rgbColor rgb="FFD9D9D9"/>
-      <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FFFF00FF"/>
-      <rgbColor rgb="FFFFFF00"/>
-      <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FF0000FF"/>
-      <rgbColor rgb="FF00CCFF"/>
-      <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FFCCFFCC"/>
-      <rgbColor rgb="FFFFFF99"/>
-      <rgbColor rgb="FF99CCFF"/>
-      <rgbColor rgb="FFFF99CC"/>
-      <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFCC99"/>
-      <rgbColor rgb="FF3366FF"/>
-      <rgbColor rgb="FF33CCCC"/>
-      <rgbColor rgb="FF99CC00"/>
-      <rgbColor rgb="FFFFCC00"/>
-      <rgbColor rgb="FFFF9900"/>
-      <rgbColor rgb="FFFF6600"/>
-      <rgbColor rgb="FF666699"/>
-      <rgbColor rgb="FF969696"/>
-      <rgbColor rgb="FF003366"/>
-      <rgbColor rgb="FF339966"/>
-      <rgbColor rgb="FF003300"/>
-      <rgbColor rgb="FF333300"/>
-      <rgbColor rgb="FF993300"/>
-      <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FF333399"/>
-      <rgbColor rgb="FF333333"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:sysClr lastClr="000000" val="windowText"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:sysClr lastClr="FFFFFF" val="window"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="44546A"/>
@@ -473,116 +381,82 @@
         <a:srgbClr val="70AD47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563C1"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954F72"/>
+        <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック Light"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Times New Roman" script="Arab"/>
+        <a:font typeface="Times New Roman" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="MoolBoran" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Times New Roman" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Arial" script="Arab"/>
+        <a:font typeface="Arial" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="DaunPenh" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Arial" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -594,177 +468,208 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="35000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
+                <a:tint val="51000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="80000">
               <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
+                <a:tint val="15000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
+                <a:tint val="94000"/>
+                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="9500"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
+                <a:alpha val="35000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot rev="0" lon="0" lat="0"/>
+            </a:camera>
+            <a:lightRig dir="t" rig="threePt">
+              <a:rot rev="1200000" lon="0" lat="0"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="40000">
               <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
+                <a:tint val="20000"/>
+                <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr summaryBelow="0"/>
+  </sheetPr>
   <dimension ref="A1:Q36"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="5.85546875" customWidth="1"/>
-    <col min="3" max="3" width="6.85546875" customWidth="1"/>
-    <col min="4" max="4" width="9.85546875" customWidth="1"/>
-    <col min="5" max="7" width="6.5703125" customWidth="1"/>
-    <col min="8" max="8" width="12.140625" customWidth="1"/>
-    <col min="9" max="9" width="4.85546875" customWidth="1"/>
-    <col min="10" max="11" width="6.5703125" customWidth="1"/>
-    <col min="12" max="12" width="5.42578125" customWidth="1"/>
-    <col min="13" max="13" width="18.85546875" customWidth="1"/>
-    <col min="14" max="17" width="6.5703125" customWidth="1"/>
-    <col min="18" max="18" width="11.5703125" customWidth="1"/>
+    <col min="1" max="1" style="13" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="14" width="5.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="15" width="6.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="15" width="9.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="15" width="6.576428571428571" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="15" width="6.576428571428571" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="15" width="6.576428571428571" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="15" width="12.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="16" width="4.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="15" width="6.576428571428571" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="15" width="6.576428571428571" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="15" width="5.433571428571429" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="15" width="18.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="15" width="6.576428571428571" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="15" width="6.576428571428571" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="15" width="6.576428571428571" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="15" width="6.576428571428571" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="3" t="s">
@@ -776,42 +681,42 @@
       <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="J1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="K1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="L1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="M1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="N1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="5" t="s">
+      <c r="O1" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="4" t="s">
+      <c r="P1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="4" t="s">
+      <c r="Q1" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="20.25">
       <c r="A2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="5">
         <v>427</v>
       </c>
-      <c r="C2">
+      <c r="C2" s="6">
         <v>6.7</v>
       </c>
       <c r="D2" s="6">
@@ -827,28 +732,28 @@
         <v>86.4</v>
       </c>
       <c r="H2" s="6">
-        <v>231000</v>
+        <v>23100000</v>
       </c>
       <c r="I2" s="7">
         <v>86</v>
       </c>
-      <c r="J2">
-        <v>0.94399999999999995</v>
-      </c>
-      <c r="K2">
-        <v>78.760000000000005</v>
+      <c r="J2" s="6">
+        <v>0.944</v>
+      </c>
+      <c r="K2" s="6">
+        <v>78.76</v>
       </c>
       <c r="L2" s="8">
         <v>60.1</v>
       </c>
       <c r="M2" s="8">
-        <v>75.581788025210102</v>
+        <v>75.5817880252101</v>
       </c>
       <c r="N2" s="6">
         <v>10.1</v>
       </c>
       <c r="O2" s="9">
-        <v>17.399999999999999</v>
+        <v>17.4</v>
       </c>
       <c r="P2" s="6">
         <v>46.7</v>
@@ -857,14 +762,14 @@
         <v>81.38</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
       <c r="A3" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="5">
         <v>181</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="5">
         <v>12</v>
       </c>
       <c r="D3" s="6">
@@ -880,22 +785,22 @@
         <v>46</v>
       </c>
       <c r="H3" s="6">
-        <v>2900000</v>
+        <v>290000000</v>
       </c>
       <c r="I3" s="7">
         <v>87</v>
       </c>
-      <c r="J3">
-        <v>0.76500000000000001</v>
-      </c>
-      <c r="K3">
+      <c r="J3" s="6">
+        <v>0.765</v>
+      </c>
+      <c r="K3" s="6">
         <v>59.57</v>
       </c>
-      <c r="L3">
+      <c r="L3" s="6">
         <v>43.6</v>
       </c>
-      <c r="M3">
-        <v>72.799435714285707</v>
+      <c r="M3" s="6">
+        <v>72.7994357142857</v>
       </c>
       <c r="N3" s="6">
         <v>5.9</v>
@@ -910,21 +815,21 @@
         <v>64.78</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
       <c r="A4" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="5">
         <v>258</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="6">
         <v>7.1</v>
       </c>
       <c r="D4" s="6">
         <v>563.54</v>
       </c>
       <c r="E4" s="6">
-        <v>78.599999999999994</v>
+        <v>78.6</v>
       </c>
       <c r="F4" s="6">
         <v>88</v>
@@ -933,29 +838,28 @@
         <v>85.9</v>
       </c>
       <c r="H4" s="6">
-        <f>2.52*1000000</f>
-        <v>2520000</v>
+        <v>252000000</v>
       </c>
       <c r="I4" s="7">
         <v>82</v>
       </c>
-      <c r="J4">
-        <v>0.92900000000000005</v>
-      </c>
-      <c r="K4">
+      <c r="J4" s="6">
+        <v>0.929</v>
+      </c>
+      <c r="K4" s="6">
         <v>88.37</v>
       </c>
-      <c r="L4">
+      <c r="L4" s="5">
         <v>50</v>
       </c>
-      <c r="M4">
-        <v>77.730482072829105</v>
+      <c r="M4" s="6">
+        <v>77.7304820728291</v>
       </c>
       <c r="N4" s="6">
-        <v>2.2000000000000002</v>
+        <v>2.2</v>
       </c>
       <c r="O4" s="6">
-        <v>38.700000000000003</v>
+        <v>38.7</v>
       </c>
       <c r="P4" s="6">
         <v>6.5</v>
@@ -964,14 +868,14 @@
         <v>84.25</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
       <c r="A5" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="5">
         <v>289</v>
       </c>
-      <c r="C5">
+      <c r="C5" s="5">
         <v>48</v>
       </c>
       <c r="D5" s="6">
@@ -983,27 +887,26 @@
       <c r="F5" s="10">
         <v>20.6</v>
       </c>
-      <c r="G5">
-        <v>32.799999999999997</v>
+      <c r="G5" s="6">
+        <v>32.8</v>
       </c>
       <c r="H5" s="10">
-        <f>420*1000</f>
-        <v>420000</v>
+        <v>42000000</v>
       </c>
       <c r="I5" s="7">
         <v>63</v>
       </c>
-      <c r="J5">
-        <v>0.76100000000000001</v>
-      </c>
-      <c r="K5">
+      <c r="J5" s="6">
+        <v>0.761</v>
+      </c>
+      <c r="K5" s="6">
         <v>62.23</v>
       </c>
-      <c r="L5">
+      <c r="L5" s="6">
         <v>28.4</v>
       </c>
-      <c r="M5">
-        <v>72.382585784313704</v>
+      <c r="M5" s="6">
+        <v>72.3825857843137</v>
       </c>
       <c r="N5" s="6">
         <v>1.4</v>
@@ -1015,23 +918,23 @@
         <v>56.1</v>
       </c>
       <c r="Q5" s="6">
-        <v>64.569999999999993</v>
-      </c>
-    </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+        <v>64.57</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
       <c r="A6" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="5">
         <v>107</v>
       </c>
-      <c r="C6">
+      <c r="C6" s="5">
         <v>22</v>
       </c>
       <c r="D6" s="6">
-        <v>77.569999999999993</v>
-      </c>
-      <c r="E6">
+        <v>77.57</v>
+      </c>
+      <c r="E6" s="6">
         <v>55.8</v>
       </c>
       <c r="F6" s="6">
@@ -1041,22 +944,22 @@
         <v>50.3</v>
       </c>
       <c r="H6" s="6">
-        <v>259000</v>
+        <v>25900000</v>
       </c>
       <c r="I6" s="7">
         <v>82</v>
       </c>
-      <c r="J6">
-        <v>0.76700000000000002</v>
-      </c>
-      <c r="K6">
+      <c r="J6" s="6">
+        <v>0.767</v>
+      </c>
+      <c r="K6" s="6">
         <v>58.04</v>
       </c>
-      <c r="L6">
+      <c r="L6" s="6">
         <v>42.4</v>
       </c>
-      <c r="M6">
-        <v>70.125614495798303</v>
+      <c r="M6" s="6">
+        <v>70.1256144957983</v>
       </c>
       <c r="N6" s="6">
         <v>4.3</v>
@@ -1071,14 +974,14 @@
         <v>63.92</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
       <c r="A7" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B7">
+      <c r="B7" s="5">
         <v>101</v>
       </c>
-      <c r="C7">
+      <c r="C7" s="5">
         <v>17</v>
       </c>
       <c r="D7" s="6">
@@ -1094,23 +997,22 @@
         <v>55.4</v>
       </c>
       <c r="H7" s="6">
-        <f>7.09*1000</f>
-        <v>7090</v>
+        <v>709000</v>
       </c>
       <c r="I7" s="7">
         <v>81</v>
       </c>
-      <c r="J7">
+      <c r="J7" s="6">
         <v>0.81</v>
       </c>
-      <c r="K7" s="11">
-        <v>68.664754803600005</v>
-      </c>
-      <c r="L7">
+      <c r="K7" s="6">
+        <v>68.6647548036</v>
+      </c>
+      <c r="L7" s="6">
         <v>46.3</v>
       </c>
-      <c r="M7" s="12">
-        <v>73.764887955182104</v>
+      <c r="M7" s="11">
+        <v>73.7648879551821</v>
       </c>
       <c r="N7" s="6">
         <v>0.9</v>
@@ -1122,17 +1024,17 @@
         <v>34.5</v>
       </c>
       <c r="Q7" s="6">
-        <v>71.849999999999994</v>
-      </c>
-    </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+        <v>71.85</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
       <c r="A8" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B8">
+      <c r="B8" s="5">
         <v>74</v>
       </c>
-      <c r="C8">
+      <c r="C8" s="5">
         <v>18</v>
       </c>
       <c r="D8" s="6">
@@ -1148,23 +1050,22 @@
         <v>33</v>
       </c>
       <c r="H8" s="6">
-        <f>14.2*1000</f>
-        <v>14200</v>
+        <v>1420000</v>
       </c>
       <c r="I8" s="7">
         <v>83</v>
       </c>
-      <c r="J8">
-        <v>0.75600000000000001</v>
-      </c>
-      <c r="K8" s="11">
-        <v>58.698913640299999</v>
-      </c>
-      <c r="L8" s="12">
+      <c r="J8" s="6">
+        <v>0.756</v>
+      </c>
+      <c r="K8" s="6">
+        <v>58.6989136403</v>
+      </c>
+      <c r="L8" s="11">
         <v>42.2</v>
       </c>
-      <c r="M8" s="12">
-        <v>70.761324509803899</v>
+      <c r="M8" s="11">
+        <v>70.7613245098039</v>
       </c>
       <c r="N8" s="6">
         <v>2.4</v>
@@ -1179,14 +1080,14 @@
         <v>65.14</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
       <c r="A9" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B9">
+      <c r="B9" s="5">
         <v>130</v>
       </c>
-      <c r="C9">
+      <c r="C9" s="5">
         <v>20</v>
       </c>
       <c r="D9" s="6">
@@ -1202,23 +1103,22 @@
         <v>46.9</v>
       </c>
       <c r="H9" s="6">
-        <f>29.7*1000</f>
-        <v>29700</v>
+        <v>2970000</v>
       </c>
       <c r="I9" s="7">
         <v>64</v>
       </c>
-      <c r="J9">
-        <v>0.75900000000000001</v>
-      </c>
-      <c r="K9" s="11">
-        <v>56.827531463699998</v>
-      </c>
-      <c r="L9">
+      <c r="J9" s="6">
+        <v>0.759</v>
+      </c>
+      <c r="K9" s="6">
+        <v>56.8275314637</v>
+      </c>
+      <c r="L9" s="6">
         <v>46.5</v>
       </c>
-      <c r="M9" s="12">
-        <v>71.549773996265202</v>
+      <c r="M9" s="11">
+        <v>71.5497739962652</v>
       </c>
       <c r="N9" s="6">
         <v>1.4</v>
@@ -1233,14 +1133,14 @@
         <v>59.24</v>
       </c>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
       <c r="A10" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B10">
+      <c r="B10" s="5">
         <v>273</v>
       </c>
-      <c r="C10">
+      <c r="C10" s="5">
         <v>11</v>
       </c>
       <c r="D10" s="6">
@@ -1256,23 +1156,22 @@
         <v>83.9</v>
       </c>
       <c r="H10" s="6">
-        <f>2.65*1000</f>
-        <v>2650</v>
+        <v>265000</v>
       </c>
       <c r="I10" s="7">
         <v>81</v>
       </c>
-      <c r="J10">
-        <v>0.90100000000000002</v>
-      </c>
-      <c r="K10">
+      <c r="J10" s="6">
+        <v>0.901</v>
+      </c>
+      <c r="K10" s="6">
         <v>76.34</v>
       </c>
-      <c r="L10" s="12">
+      <c r="L10" s="11">
         <v>62.5</v>
       </c>
-      <c r="M10" s="12">
-        <v>81.239405182072801</v>
+      <c r="M10" s="11">
+        <v>81.2394051820728</v>
       </c>
       <c r="N10" s="6">
         <v>0</v>
@@ -1287,21 +1186,21 @@
         <v>87.63</v>
       </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5">
       <c r="A11" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B11">
+      <c r="B11" s="5">
         <v>196</v>
       </c>
-      <c r="C11">
+      <c r="C11" s="5">
         <v>12</v>
       </c>
       <c r="D11" s="6">
         <v>665.88</v>
       </c>
       <c r="E11" s="6">
-        <v>36.200000000000003</v>
+        <v>36.2</v>
       </c>
       <c r="F11" s="6">
         <v>75.2</v>
@@ -1310,29 +1209,28 @@
         <v>82</v>
       </c>
       <c r="H11" s="6">
-        <f>202*1000</f>
-        <v>202000</v>
+        <v>20200000</v>
       </c>
       <c r="I11" s="7">
         <v>78</v>
       </c>
-      <c r="J11">
-        <v>0.94699999999999995</v>
-      </c>
-      <c r="K11">
-        <v>80.569999999999993</v>
-      </c>
-      <c r="L11" s="12">
+      <c r="J11" s="6">
+        <v>0.947</v>
+      </c>
+      <c r="K11" s="6">
+        <v>80.57</v>
+      </c>
+      <c r="L11" s="11">
         <v>62.4</v>
       </c>
-      <c r="M11" s="12">
-        <v>82.178738935574202</v>
+      <c r="M11" s="11">
+        <v>82.1787389355742</v>
       </c>
       <c r="N11" s="6">
         <v>0.1</v>
       </c>
       <c r="O11" s="6">
-        <v>32.700000000000003</v>
+        <v>32.7</v>
       </c>
       <c r="P11" s="6">
         <v>47.6</v>
@@ -1341,14 +1239,14 @@
         <v>88.73</v>
       </c>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5">
       <c r="A12" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B12">
+      <c r="B12" s="5">
         <v>249</v>
       </c>
-      <c r="C12">
+      <c r="C12" s="5">
         <v>83</v>
       </c>
       <c r="D12" s="6">
@@ -1364,23 +1262,22 @@
         <v>12.5</v>
       </c>
       <c r="H12" s="6">
-        <f>127*1000</f>
-        <v>127000</v>
+        <v>12700000</v>
       </c>
       <c r="I12" s="7">
         <v>35</v>
       </c>
-      <c r="J12">
-        <v>0.64500000000000002</v>
-      </c>
-      <c r="K12">
+      <c r="J12" s="6">
+        <v>0.645</v>
+      </c>
+      <c r="K12" s="6">
         <v>53.57</v>
       </c>
-      <c r="L12" s="12">
-        <v>18.899999999999999</v>
-      </c>
-      <c r="M12" s="12">
-        <v>60.317517997198898</v>
+      <c r="L12" s="11">
+        <v>18.9</v>
+      </c>
+      <c r="M12" s="11">
+        <v>60.3175179971989</v>
       </c>
       <c r="N12" s="6">
         <v>1.9</v>
@@ -1395,21 +1292,21 @@
         <v>62.48</v>
       </c>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="19.5">
       <c r="A13" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B13">
+      <c r="B13" s="5">
         <v>120</v>
       </c>
-      <c r="C13">
+      <c r="C13" s="6">
         <v>7.9</v>
       </c>
       <c r="D13" s="6">
         <v>35.01</v>
       </c>
       <c r="E13" s="6">
-        <v>40.200000000000003</v>
+        <v>40.2</v>
       </c>
       <c r="F13" s="6">
         <v>96</v>
@@ -1418,23 +1315,22 @@
         <v>88.3</v>
       </c>
       <c r="H13" s="6">
-        <f>2.57*1000</f>
-        <v>2570</v>
+        <v>257000</v>
       </c>
       <c r="I13" s="7">
         <v>64</v>
       </c>
-      <c r="J13">
-        <v>0.95499999999999996</v>
-      </c>
-      <c r="K13">
+      <c r="J13" s="6">
+        <v>0.955</v>
+      </c>
+      <c r="K13" s="6">
         <v>79.63</v>
       </c>
-      <c r="L13" s="12">
+      <c r="L13" s="11">
         <v>57.4</v>
       </c>
-      <c r="M13" s="12">
-        <v>80.662983193277299</v>
+      <c r="M13" s="11">
+        <v>80.6629831932773</v>
       </c>
       <c r="N13" s="6">
         <v>0</v>
@@ -1443,20 +1339,20 @@
         <v>0.5</v>
       </c>
       <c r="P13" s="6">
-        <v>65.599999999999994</v>
+        <v>65.6</v>
       </c>
       <c r="Q13" s="6">
         <v>85.75</v>
       </c>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
       <c r="A14" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B14">
+      <c r="B14" s="5">
         <v>283</v>
       </c>
-      <c r="C14">
+      <c r="C14" s="5">
         <v>13</v>
       </c>
       <c r="D14" s="6">
@@ -1466,35 +1362,34 @@
         <v>44.2</v>
       </c>
       <c r="F14" s="6">
-        <v>78.900000000000006</v>
+        <v>78.9</v>
       </c>
       <c r="G14" s="6">
         <v>82.5</v>
       </c>
       <c r="H14" s="6">
-        <f>18.6*1000</f>
-        <v>18600</v>
+        <v>1860000</v>
       </c>
       <c r="I14" s="7">
         <v>92</v>
       </c>
-      <c r="J14">
-        <v>0.91900000000000004</v>
-      </c>
-      <c r="K14">
+      <c r="J14" s="6">
+        <v>0.919</v>
+      </c>
+      <c r="K14" s="6">
         <v>77.72</v>
       </c>
       <c r="L14" s="8">
         <v>57.2</v>
       </c>
       <c r="M14" s="8">
-        <v>79.581691176470599</v>
+        <v>79.5816911764706</v>
       </c>
       <c r="N14" s="6">
         <v>0.2</v>
       </c>
       <c r="O14" s="6">
-        <v>68.400000000000006</v>
+        <v>68.4</v>
       </c>
       <c r="P14" s="6">
         <v>12.1</v>
@@ -1503,21 +1398,21 @@
         <v>78.45</v>
       </c>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="20.25">
       <c r="A15" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B15">
+      <c r="B15" s="5">
         <v>98</v>
       </c>
-      <c r="C15">
+      <c r="C15" s="5">
         <v>22</v>
       </c>
       <c r="D15" s="6">
         <v>22.43</v>
       </c>
       <c r="E15" s="6">
-        <v>37.200000000000003</v>
+        <v>37.2</v>
       </c>
       <c r="F15" s="6">
         <v>30</v>
@@ -1526,16 +1421,15 @@
         <v>26.2</v>
       </c>
       <c r="H15" s="6">
-        <f>7.23*1000</f>
-        <v>7230</v>
+        <v>723000</v>
       </c>
       <c r="I15" s="7">
         <v>28</v>
       </c>
-      <c r="J15">
-        <v>0.60099999999999998</v>
-      </c>
-      <c r="K15">
+      <c r="J15" s="6">
+        <v>0.601</v>
+      </c>
+      <c r="K15" s="6">
         <v>51.09</v>
       </c>
       <c r="L15" s="8">
@@ -1557,14 +1451,14 @@
         <v>55.4</v>
       </c>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="19.5">
       <c r="A16" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B16">
+      <c r="B16" s="5">
         <v>214</v>
       </c>
-      <c r="C16">
+      <c r="C16" s="5">
         <v>20</v>
       </c>
       <c r="D16" s="6">
@@ -1574,35 +1468,34 @@
         <v>44.2</v>
       </c>
       <c r="F16" s="6">
-        <v>34.200000000000003</v>
+        <v>34.2</v>
       </c>
       <c r="G16" s="6">
         <v>40.9</v>
       </c>
       <c r="H16" s="6">
-        <f>186*1000</f>
-        <v>186000</v>
-      </c>
-      <c r="I16" s="13">
+        <v>18600000</v>
+      </c>
+      <c r="I16" s="12">
         <v>81</v>
       </c>
-      <c r="J16">
-        <v>0.77900000000000003</v>
-      </c>
-      <c r="K16">
+      <c r="J16" s="6">
+        <v>0.779</v>
+      </c>
+      <c r="K16" s="6">
         <v>59.15</v>
       </c>
-      <c r="L16" s="12">
+      <c r="L16" s="11">
         <v>45.5</v>
       </c>
-      <c r="M16" s="12">
-        <v>70.204482492997201</v>
+      <c r="M16" s="11">
+        <v>70.2044824929972</v>
       </c>
       <c r="N16" s="6">
         <v>2.7</v>
       </c>
       <c r="O16" s="6">
-        <v>33.799999999999997</v>
+        <v>33.8</v>
       </c>
       <c r="P16" s="6">
         <v>55</v>
@@ -1611,14 +1504,14 @@
         <v>71.45</v>
       </c>
     </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="19.5">
       <c r="A17" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B17">
+      <c r="B17" s="5">
         <v>104</v>
       </c>
-      <c r="C17">
+      <c r="C17" s="5">
         <v>35</v>
       </c>
       <c r="D17" s="6">
@@ -1634,22 +1527,21 @@
         <v>28.6</v>
       </c>
       <c r="H17" s="6">
-        <f>1.54*1000</f>
-        <v>1540</v>
+        <v>154000</v>
       </c>
       <c r="I17" s="7">
         <v>64</v>
       </c>
-      <c r="J17">
-        <v>0.68600000000000005</v>
-      </c>
-      <c r="K17">
+      <c r="J17" s="6">
+        <v>0.686</v>
+      </c>
+      <c r="K17" s="6">
         <v>55.97</v>
       </c>
-      <c r="L17" s="12">
+      <c r="L17" s="11">
         <v>28.4</v>
       </c>
-      <c r="M17" s="12">
+      <c r="M17" s="11">
         <v>68.9807887254902</v>
       </c>
       <c r="N17" s="6">
@@ -1659,24 +1551,24 @@
         <v>12.9</v>
       </c>
       <c r="P17" s="6">
-        <v>67.400000000000006</v>
+        <v>67.4</v>
       </c>
       <c r="Q17" s="6">
         <v>70.47</v>
       </c>
     </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="19.5">
       <c r="A18" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B18">
+      <c r="B18" s="5">
         <v>66</v>
       </c>
-      <c r="C18">
+      <c r="C18" s="5">
         <v>70</v>
       </c>
       <c r="D18" s="6">
-        <v>2.4700000000000002</v>
+        <v>2.47</v>
       </c>
       <c r="E18" s="6">
         <v>33</v>
@@ -1688,23 +1580,22 @@
         <v>15.2</v>
       </c>
       <c r="H18" s="6">
-        <f>96.5*1000</f>
-        <v>96500</v>
+        <v>9650000</v>
       </c>
       <c r="I18" s="7">
         <v>53</v>
       </c>
-      <c r="J18">
-        <v>0.53900000000000003</v>
-      </c>
-      <c r="K18">
+      <c r="J18" s="6">
+        <v>0.539</v>
+      </c>
+      <c r="K18" s="6">
         <v>43.02</v>
       </c>
-      <c r="L18" s="12">
+      <c r="L18" s="11">
         <v>28.3</v>
       </c>
-      <c r="M18" s="12">
-        <v>54.233591129785196</v>
+      <c r="M18" s="11">
+        <v>54.2335911297852</v>
       </c>
       <c r="N18" s="6">
         <v>6.2</v>
@@ -1713,27 +1604,27 @@
         <v>23.7</v>
       </c>
       <c r="P18" s="6">
-        <v>75.900000000000006</v>
+        <v>75.9</v>
       </c>
       <c r="Q18" s="6">
         <v>45.68</v>
       </c>
     </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="19.5">
       <c r="A19" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B19">
+      <c r="B19" s="5">
         <v>102</v>
       </c>
-      <c r="C19">
+      <c r="C19" s="5">
         <v>63</v>
       </c>
       <c r="D19" s="6">
         <v>219.79</v>
       </c>
       <c r="E19" s="6">
-        <v>39.700000000000003</v>
+        <v>39.7</v>
       </c>
       <c r="F19" s="6">
         <v>5.7</v>
@@ -1742,22 +1633,22 @@
         <v>11.4</v>
       </c>
       <c r="H19" s="6">
-        <v>63.2</v>
+        <v>6320</v>
       </c>
       <c r="I19" s="7">
         <v>37</v>
       </c>
-      <c r="J19">
-        <v>0.55700000000000005</v>
-      </c>
-      <c r="K19">
+      <c r="J19" s="6">
+        <v>0.557</v>
+      </c>
+      <c r="K19" s="6">
         <v>44.13</v>
       </c>
-      <c r="L19" s="12">
+      <c r="L19" s="11">
         <v>24.6</v>
       </c>
-      <c r="M19" s="12">
-        <v>59.338261764705898</v>
+      <c r="M19" s="11">
+        <v>59.3382617647059</v>
       </c>
       <c r="N19" s="6">
         <v>0.9</v>
@@ -1772,14 +1663,14 @@
         <v>53.59</v>
       </c>
     </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="20.25">
       <c r="A20" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B20">
+      <c r="B20" s="5">
         <v>84</v>
       </c>
-      <c r="C20">
+      <c r="C20" s="5">
         <v>13</v>
       </c>
       <c r="D20" s="6">
@@ -1795,23 +1686,22 @@
         <v>49</v>
       </c>
       <c r="H20" s="6">
-        <f>24.4*1000</f>
-        <v>24400</v>
+        <v>2440000</v>
       </c>
       <c r="I20" s="7">
         <v>69</v>
       </c>
-      <c r="J20">
-        <v>0.67500000000000004</v>
-      </c>
-      <c r="K20" s="11">
-        <v>63.558505842000002</v>
-      </c>
-      <c r="L20" s="12">
+      <c r="J20" s="6">
+        <v>0.675</v>
+      </c>
+      <c r="K20" s="6">
+        <v>63.558505842</v>
+      </c>
+      <c r="L20" s="11">
         <v>50.5</v>
       </c>
-      <c r="M20" s="12">
-        <v>63.999157492997199</v>
+      <c r="M20" s="11">
+        <v>63.9991574929972</v>
       </c>
       <c r="N20" s="6">
         <v>0.1</v>
@@ -1826,14 +1716,14 @@
         <v>71.3</v>
       </c>
     </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="19.5">
       <c r="A21" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B21">
+      <c r="B21" s="5">
         <v>110</v>
       </c>
-      <c r="C21">
+      <c r="C21" s="5">
         <v>31</v>
       </c>
       <c r="D21" s="6">
@@ -1849,52 +1739,51 @@
         <v>43.1</v>
       </c>
       <c r="H21" s="6">
-        <f>224*1000</f>
-        <v>224000</v>
-      </c>
-      <c r="I21" s="13">
+        <v>22400000</v>
+      </c>
+      <c r="I21" s="12">
         <v>79</v>
       </c>
-      <c r="J21">
-        <v>0.77700000000000002</v>
-      </c>
-      <c r="K21">
+      <c r="J21" s="6">
+        <v>0.777</v>
+      </c>
+      <c r="K21" s="6">
         <v>60.81</v>
       </c>
-      <c r="L21">
-        <v>39.799999999999997</v>
-      </c>
-      <c r="M21" s="12">
-        <v>71.928091386554598</v>
+      <c r="L21" s="6">
+        <v>39.8</v>
+      </c>
+      <c r="M21" s="11">
+        <v>71.9280913865546</v>
       </c>
       <c r="N21" s="6">
-        <v>4.4000000000000004</v>
+        <v>4.4</v>
       </c>
       <c r="O21" s="6">
         <v>56.5</v>
       </c>
       <c r="P21" s="6">
-        <v>18.399999999999999</v>
+        <v>18.4</v>
       </c>
       <c r="Q21" s="6">
-        <v>68.650000000000006</v>
-      </c>
-    </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.25">
+        <v>68.65</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="19.5">
       <c r="A22" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B22">
+      <c r="B22" s="5">
         <v>152</v>
       </c>
-      <c r="C22">
+      <c r="C22" s="5">
         <v>19</v>
       </c>
       <c r="D22" s="6">
         <v>147.96</v>
       </c>
       <c r="E22" s="6">
-        <v>35.799999999999997</v>
+        <v>35.8</v>
       </c>
       <c r="F22" s="6">
         <v>25.9</v>
@@ -1903,23 +1792,22 @@
         <v>31.1</v>
       </c>
       <c r="H22" s="6">
-        <f>37.7*1000</f>
-        <v>37700</v>
+        <v>3770000</v>
       </c>
       <c r="I22" s="7">
         <v>48</v>
       </c>
-      <c r="J22">
-        <v>0.71799999999999997</v>
-      </c>
-      <c r="K22">
+      <c r="J22" s="6">
+        <v>0.718</v>
+      </c>
+      <c r="K22" s="6">
         <v>56.75</v>
       </c>
-      <c r="L22">
+      <c r="L22" s="6">
         <v>28.9</v>
       </c>
-      <c r="M22" s="12">
-        <v>66.638341129785204</v>
+      <c r="M22" s="11">
+        <v>66.6383411297852</v>
       </c>
       <c r="N22" s="6">
         <v>1.4</v>
@@ -1934,14 +1822,14 @@
         <v>66.08</v>
       </c>
     </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="19.5">
       <c r="A23" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B23">
+      <c r="B23" s="5">
         <v>151</v>
       </c>
-      <c r="C23">
+      <c r="C23" s="5">
         <v>23</v>
       </c>
       <c r="D23" s="6">
@@ -1950,30 +1838,29 @@
       <c r="E23" s="6">
         <v>37</v>
       </c>
-      <c r="F23">
+      <c r="F23" s="6">
         <v>40.4</v>
       </c>
       <c r="G23" s="6">
         <v>53</v>
       </c>
       <c r="H23" s="6">
-        <f>77.6*1000</f>
-        <v>77600</v>
+        <v>7760000</v>
       </c>
       <c r="I23" s="7">
         <v>60</v>
       </c>
-      <c r="J23">
+      <c r="J23" s="6">
         <v>0.88</v>
       </c>
-      <c r="K23">
-        <v>70.319999999999993</v>
-      </c>
-      <c r="L23">
+      <c r="K23" s="6">
+        <v>70.32</v>
+      </c>
+      <c r="L23" s="6">
         <v>50.6</v>
       </c>
-      <c r="M23" s="12">
-        <v>80.536741316526602</v>
+      <c r="M23" s="11">
+        <v>80.5367413165266</v>
       </c>
       <c r="N23" s="6">
         <v>0.9</v>
@@ -1988,15 +1875,15 @@
         <v>80.02</v>
       </c>
     </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="19.5">
       <c r="A24" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B24">
+      <c r="B24" s="5">
         <v>187</v>
       </c>
-      <c r="C24">
-        <v>8.3000000000000007</v>
+      <c r="C24" s="6">
+        <v>8.3</v>
       </c>
       <c r="D24" s="6">
         <v>38.68</v>
@@ -2005,35 +1892,34 @@
         <v>35</v>
       </c>
       <c r="F24" s="6">
-        <v>78.099999999999994</v>
+        <v>78.1</v>
       </c>
       <c r="G24" s="6">
-        <v>76.599999999999994</v>
+        <v>76.6</v>
       </c>
       <c r="H24" s="6">
-        <f>10.2*1000</f>
-        <v>10200</v>
+        <v>1020000</v>
       </c>
       <c r="I24" s="7">
         <v>67</v>
       </c>
-      <c r="J24">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="K24">
-        <v>74.209999999999994</v>
-      </c>
-      <c r="L24">
+      <c r="J24" s="6">
+        <v>0.864</v>
+      </c>
+      <c r="K24" s="6">
+        <v>74.21</v>
+      </c>
+      <c r="L24" s="6">
         <v>50.4</v>
       </c>
-      <c r="M24" s="12">
-        <v>79.226426890756301</v>
+      <c r="M24" s="11">
+        <v>79.2264268907563</v>
       </c>
       <c r="N24" s="6">
         <v>0.2</v>
       </c>
       <c r="O24" s="6">
-        <v>36.200000000000003</v>
+        <v>36.2</v>
       </c>
       <c r="P24" s="6">
         <v>39</v>
@@ -2042,21 +1928,21 @@
         <v>85.22</v>
       </c>
     </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="19.5">
       <c r="A25" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B25">
+      <c r="B25" s="5">
         <v>193</v>
       </c>
-      <c r="C25">
+      <c r="C25" s="5">
         <v>12</v>
       </c>
       <c r="D25" s="6">
         <v>1942.54</v>
       </c>
       <c r="E25" s="6">
-        <v>69.599999999999994</v>
+        <v>69.6</v>
       </c>
       <c r="F25" s="6">
         <v>48.8</v>
@@ -2065,23 +1951,22 @@
         <v>50.6</v>
       </c>
       <c r="H25" s="6">
-        <f>6.52*1000000</f>
-        <v>6520000</v>
+        <v>652000000</v>
       </c>
       <c r="I25" s="7">
         <v>75</v>
       </c>
-      <c r="J25">
-        <v>0.82399999999999995</v>
-      </c>
-      <c r="K25">
+      <c r="J25" s="6">
+        <v>0.824</v>
+      </c>
+      <c r="K25" s="6">
         <v>59.1</v>
       </c>
-      <c r="L25">
+      <c r="L25" s="6">
         <v>37.5</v>
       </c>
-      <c r="M25" s="12">
-        <v>74.074165406162507</v>
+      <c r="M25" s="11">
+        <v>74.0741654061625</v>
       </c>
       <c r="N25" s="6">
         <v>11</v>
@@ -2096,14 +1981,14 @@
         <v>72.03</v>
       </c>
     </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="19.5">
       <c r="A26" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B26">
+      <c r="B26" s="5">
         <v>52</v>
       </c>
-      <c r="C26">
+      <c r="C26" s="5">
         <v>62</v>
       </c>
       <c r="D26" s="6">
@@ -2113,7 +1998,7 @@
         <v>58</v>
       </c>
       <c r="F26" s="6">
-        <v>32.799999999999997</v>
+        <v>32.8</v>
       </c>
       <c r="G26" s="6">
         <v>42.4</v>
@@ -2124,17 +2009,17 @@
       <c r="I26" s="7">
         <v>85</v>
       </c>
-      <c r="J26">
-        <v>0.85399999999999998</v>
-      </c>
-      <c r="K26">
+      <c r="J26" s="6">
+        <v>0.854</v>
+      </c>
+      <c r="K26" s="6">
         <v>58.59</v>
       </c>
-      <c r="L26">
+      <c r="L26" s="6">
         <v>37.9</v>
       </c>
-      <c r="M26" s="12">
-        <v>66.562038712757797</v>
+      <c r="M26" s="11">
+        <v>66.5620387127578</v>
       </c>
       <c r="N26" s="6">
         <v>18.3</v>
@@ -2146,24 +2031,24 @@
         <v>80.8</v>
       </c>
       <c r="Q26" s="6">
-        <v>67.599999999999994</v>
-      </c>
-    </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.25">
+        <v>67.6</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="19.5">
       <c r="A27" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B27">
+      <c r="B27" s="5">
         <v>82</v>
       </c>
-      <c r="C27">
+      <c r="C27" s="5">
         <v>19</v>
       </c>
       <c r="D27" s="6">
         <v>58.18</v>
       </c>
       <c r="E27" s="6">
-        <v>78.099999999999994</v>
+        <v>78.1</v>
       </c>
       <c r="F27" s="6">
         <v>69.2</v>
@@ -2172,22 +2057,22 @@
         <v>77</v>
       </c>
       <c r="H27" s="6">
-        <v>201</v>
+        <v>20100</v>
       </c>
       <c r="I27" s="7">
         <v>100</v>
       </c>
-      <c r="J27">
-        <v>0.93799999999999994</v>
-      </c>
-      <c r="K27">
+      <c r="J27" s="6">
+        <v>0.938</v>
+      </c>
+      <c r="K27" s="6">
         <v>79.05</v>
       </c>
-      <c r="L27">
+      <c r="L27" s="6">
         <v>50.9</v>
       </c>
-      <c r="M27" s="12">
-        <v>71.719216660830995</v>
+      <c r="M27" s="11">
+        <v>71.719216660831</v>
       </c>
       <c r="N27" s="6">
         <v>0</v>
@@ -2202,18 +2087,18 @@
         <v>83.47</v>
       </c>
     </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="19.5">
       <c r="A28" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="B28">
+      <c r="B28" s="5">
         <v>66</v>
       </c>
-      <c r="C28">
+      <c r="C28" s="5">
         <v>18</v>
       </c>
       <c r="D28" s="6">
-        <v>37.479999999999997</v>
+        <v>37.48</v>
       </c>
       <c r="E28" s="6">
         <v>35.6</v>
@@ -2225,23 +2110,22 @@
         <v>59</v>
       </c>
       <c r="H28" s="6">
-        <f>6.1*1000</f>
-        <v>6100</v>
+        <v>610000</v>
       </c>
       <c r="I28" s="7">
         <v>54</v>
       </c>
-      <c r="J28">
+      <c r="J28" s="6">
         <v>0.86</v>
       </c>
-      <c r="K28">
+      <c r="K28" s="6">
         <v>70.56</v>
       </c>
-      <c r="L28">
+      <c r="L28" s="5">
         <v>60</v>
       </c>
-      <c r="M28" s="12">
-        <v>78.661754140406202</v>
+      <c r="M28" s="11">
+        <v>78.6617541404062</v>
       </c>
       <c r="N28" s="6">
         <v>0.2</v>
@@ -2250,20 +2134,20 @@
         <v>40.1</v>
       </c>
       <c r="P28" s="6">
-        <v>39.299999999999997</v>
+        <v>39.3</v>
       </c>
       <c r="Q28" s="6">
         <v>82.71</v>
       </c>
     </row>
-    <row r="29" spans="1:17" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="19.5">
       <c r="A29" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B29">
+      <c r="B29" s="5">
         <v>216</v>
       </c>
-      <c r="C29">
+      <c r="C29" s="5">
         <v>29</v>
       </c>
       <c r="D29" s="6">
@@ -2279,23 +2163,22 @@
         <v>28.1</v>
       </c>
       <c r="H29" s="6">
-        <f>23.9*1000</f>
-        <v>23900</v>
+        <v>2390000</v>
       </c>
       <c r="I29" s="7">
         <v>68</v>
       </c>
-      <c r="J29">
-        <v>0.70899999999999996</v>
-      </c>
-      <c r="K29">
+      <c r="J29" s="6">
+        <v>0.709</v>
+      </c>
+      <c r="K29" s="6">
         <v>56.69</v>
       </c>
-      <c r="L29">
-        <v>37.200000000000003</v>
-      </c>
-      <c r="M29" s="12">
-        <v>63.722764005602201</v>
+      <c r="L29" s="6">
+        <v>37.2</v>
+      </c>
+      <c r="M29" s="11">
+        <v>63.7227640056022</v>
       </c>
       <c r="N29" s="6">
         <v>5.4</v>
@@ -2304,24 +2187,24 @@
         <v>14.1</v>
       </c>
       <c r="P29" s="6">
-        <v>79.400000000000006</v>
+        <v>79.4</v>
       </c>
       <c r="Q29" s="6">
         <v>70.2</v>
       </c>
     </row>
-    <row r="30" spans="1:17" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="19.5">
       <c r="A30" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="B30">
+      <c r="B30" s="5">
         <v>109</v>
       </c>
-      <c r="C30">
+      <c r="C30" s="5">
         <v>27</v>
       </c>
       <c r="D30" s="6">
-        <v>626.79999999999995</v>
+        <v>626.8</v>
       </c>
       <c r="E30" s="6">
         <v>41.6</v>
@@ -2333,23 +2216,22 @@
         <v>73.3</v>
       </c>
       <c r="H30" s="6">
-        <f>12.8*1000</f>
-        <v>12800</v>
+        <v>1280000</v>
       </c>
       <c r="I30" s="7">
         <v>81</v>
       </c>
-      <c r="J30">
-        <v>0.91600000000000004</v>
-      </c>
-      <c r="K30">
+      <c r="J30" s="6">
+        <v>0.916</v>
+      </c>
+      <c r="K30" s="6">
         <v>73.52</v>
       </c>
-      <c r="L30">
+      <c r="L30" s="6">
         <v>46.9</v>
       </c>
-      <c r="M30" s="12">
-        <v>77.895219164332403</v>
+      <c r="M30" s="11">
+        <v>77.8952191643324</v>
       </c>
       <c r="N30" s="6">
         <v>0.2</v>
@@ -2358,58 +2240,57 @@
         <v>64.5</v>
       </c>
       <c r="P30" s="6">
-        <v>16.899999999999999</v>
+        <v>16.9</v>
       </c>
       <c r="Q30" s="6">
-        <v>78.760000000000005</v>
-      </c>
-    </row>
-    <row r="31" spans="1:17" x14ac:dyDescent="0.25">
+        <v>78.76</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="19.5">
       <c r="A31" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B31">
+      <c r="B31" s="5">
         <v>253</v>
       </c>
-      <c r="C31">
-        <v>9.6999999999999993</v>
+      <c r="C31" s="6">
+        <v>9.7</v>
       </c>
       <c r="D31" s="6">
         <v>231.91</v>
       </c>
       <c r="E31" s="6">
-        <v>32.799999999999997</v>
+        <v>32.8</v>
       </c>
       <c r="F31" s="6">
         <v>74</v>
       </c>
       <c r="G31" s="6">
-        <v>78.099999999999994</v>
+        <v>78.1</v>
       </c>
       <c r="H31" s="6">
-        <f>46.4*1000</f>
-        <v>46400</v>
+        <v>4640000</v>
       </c>
       <c r="I31" s="7">
         <v>81</v>
       </c>
-      <c r="J31">
-        <v>0.90400000000000003</v>
-      </c>
-      <c r="K31">
+      <c r="J31" s="6">
+        <v>0.904</v>
+      </c>
+      <c r="K31" s="6">
         <v>75.44</v>
       </c>
-      <c r="L31">
+      <c r="L31" s="6">
         <v>56.6</v>
       </c>
-      <c r="M31">
-        <v>79.897383182503802</v>
+      <c r="M31" s="6">
+        <v>79.8973831825038</v>
       </c>
       <c r="N31" s="6">
         <v>0.1</v>
       </c>
       <c r="O31" s="6">
-        <v>37.200000000000003</v>
+        <v>37.2</v>
       </c>
       <c r="P31" s="6">
         <v>52.4</v>
@@ -2418,14 +2299,14 @@
         <v>85.87</v>
       </c>
     </row>
-    <row r="32" spans="1:17" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="19.5">
       <c r="A32" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="B32">
+      <c r="B32" s="5">
         <v>135</v>
       </c>
-      <c r="C32">
+      <c r="C32" s="6">
         <v>5.6</v>
       </c>
       <c r="D32" s="6">
@@ -2441,23 +2322,22 @@
         <v>93.1</v>
       </c>
       <c r="H32" s="6">
-        <f>333*1000</f>
-        <v>333000</v>
+        <v>33300000</v>
       </c>
       <c r="I32" s="7">
         <v>88</v>
       </c>
-      <c r="J32">
-        <v>0.94499999999999995</v>
-      </c>
-      <c r="K32">
+      <c r="J32" s="6">
+        <v>0.945</v>
+      </c>
+      <c r="K32" s="6">
         <v>83.11</v>
       </c>
-      <c r="L32">
+      <c r="L32" s="6">
         <v>72.7</v>
       </c>
-      <c r="M32">
-        <v>85.189279438698605</v>
+      <c r="M32" s="6">
+        <v>85.1892794386986</v>
       </c>
       <c r="N32" s="6">
         <v>0.9</v>
@@ -2472,14 +2352,14 @@
         <v>89.44</v>
       </c>
     </row>
-    <row r="33" spans="1:17" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18.75">
       <c r="A33" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B33">
+      <c r="B33" s="5">
         <v>141</v>
       </c>
-      <c r="C33">
+      <c r="C33" s="5">
         <v>27</v>
       </c>
       <c r="D33" s="6">
@@ -2495,23 +2375,22 @@
         <v>43.8</v>
       </c>
       <c r="H33" s="6">
-        <f>122*1000</f>
-        <v>122000</v>
+        <v>12200000</v>
       </c>
       <c r="I33" s="7">
         <v>52</v>
       </c>
-      <c r="J33">
-        <v>0.77700000000000002</v>
-      </c>
-      <c r="K33">
+      <c r="J33" s="6">
+        <v>0.777</v>
+      </c>
+      <c r="K33" s="6">
         <v>60.51</v>
       </c>
-      <c r="L33" s="12">
+      <c r="L33" s="11">
         <v>38.1</v>
       </c>
-      <c r="M33" s="12">
-        <v>74.125647992530403</v>
+      <c r="M33" s="11">
+        <v>74.1256479925304</v>
       </c>
       <c r="N33" s="6">
         <v>1.3</v>
@@ -2526,14 +2405,14 @@
         <v>73.3</v>
       </c>
     </row>
-    <row r="34" spans="1:17" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18.75">
       <c r="A34" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="B34">
+      <c r="B34" s="5">
         <v>29</v>
       </c>
-      <c r="C34">
+      <c r="C34" s="5">
         <v>44</v>
       </c>
       <c r="D34" s="6">
@@ -2554,17 +2433,17 @@
       <c r="I34" s="7">
         <v>87</v>
       </c>
-      <c r="J34">
+      <c r="J34" s="6">
         <v>0.89</v>
       </c>
-      <c r="K34">
+      <c r="K34" s="6">
         <v>67.31</v>
       </c>
-      <c r="L34" s="12">
+      <c r="L34" s="11">
         <v>52.4</v>
       </c>
-      <c r="M34" s="12">
-        <v>68.835716900093402</v>
+      <c r="M34" s="11">
+        <v>68.8357169000934</v>
       </c>
       <c r="N34" s="6">
         <v>11.9</v>
@@ -2579,46 +2458,45 @@
         <v>75.78</v>
       </c>
     </row>
-    <row r="35" spans="1:17" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="18.75">
       <c r="A35" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B35">
+      <c r="B35" s="5">
         <v>240</v>
       </c>
-      <c r="C35">
+      <c r="C35" s="5">
         <v>10</v>
       </c>
       <c r="D35" s="6">
         <v>335.36</v>
       </c>
       <c r="E35" s="6">
-        <v>36.799999999999997</v>
+        <v>36.8</v>
       </c>
       <c r="F35" s="6">
-        <v>78.599999999999994</v>
+        <v>78.6</v>
       </c>
       <c r="G35" s="6">
         <v>83.9</v>
       </c>
       <c r="H35" s="6">
-        <f>5.25*1000</f>
-        <v>5250</v>
+        <v>525000</v>
       </c>
       <c r="I35" s="7">
         <v>84</v>
       </c>
-      <c r="J35">
-        <v>0.93200000000000005</v>
-      </c>
-      <c r="K35">
-        <v>79.599999999999994</v>
+      <c r="J35" s="6">
+        <v>0.932</v>
+      </c>
+      <c r="K35" s="6">
+        <v>79.6</v>
       </c>
       <c r="L35" s="8">
         <v>77.7</v>
       </c>
       <c r="M35" s="8">
-        <v>80.550105381383304</v>
+        <v>80.5501053813833</v>
       </c>
       <c r="N35" s="6">
         <v>0.4</v>
@@ -2629,18 +2507,18 @@
       <c r="P35" s="6">
         <v>71.7</v>
       </c>
-      <c r="Q35">
+      <c r="Q35" s="6">
         <v>89.31</v>
       </c>
     </row>
-    <row r="36" spans="1:17" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="18.75">
       <c r="A36" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="B36">
+      <c r="B36" s="5">
         <v>692</v>
       </c>
-      <c r="C36">
+      <c r="C36" s="6">
         <v>7.7</v>
       </c>
       <c r="D36" s="6">
@@ -2656,23 +2534,22 @@
         <v>76.8</v>
       </c>
       <c r="H36" s="6">
-        <f>1.71*1000000</f>
-        <v>1710000</v>
+        <v>171000000</v>
       </c>
       <c r="I36" s="7">
         <v>83</v>
       </c>
-      <c r="J36">
-        <v>0.92600000000000005</v>
-      </c>
-      <c r="K36">
-        <v>77.150000000000006</v>
-      </c>
-      <c r="L36" s="12">
+      <c r="J36" s="6">
+        <v>0.926</v>
+      </c>
+      <c r="K36" s="6">
+        <v>77.15</v>
+      </c>
+      <c r="L36" s="11">
         <v>51.1</v>
       </c>
-      <c r="M36" s="12">
-        <v>74.551987605042001</v>
+      <c r="M36" s="11">
+        <v>74.551987605042</v>
       </c>
       <c r="N36" s="6">
         <v>0.5</v>
@@ -2688,7 +2565,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>